<commit_message>
eff, af, and bev demand
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/BY_Trans.xlsx
+++ b/VerveStacks_ZAF_grids_kan/BY_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D1EB1B-B45C-4149-AEE2-7B3180C9E8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C66D1A-E30F-4211-9B97-97CB335D82CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="misc." sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="62">
   <si>
     <t>attribute</t>
   </si>
@@ -205,13 +205,28 @@
   </si>
   <si>
     <t>*_hydro_ps*</t>
+  </si>
+  <si>
+    <t>~TFM_UPD</t>
+  </si>
+  <si>
+    <t>Eff</t>
+  </si>
+  <si>
+    <t>*.9</t>
+  </si>
+  <si>
+    <t>ep_coal_super*</t>
+  </si>
+  <si>
+    <t>these are aircooled plants</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,6 +246,15 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -276,11 +300,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
@@ -617,7 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{982CB9B3-DA63-443B-9AA5-BEE16CBC2D59}">
-  <dimension ref="B3:L25"/>
+  <dimension ref="B3:L30"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.53125" bestFit="1" customWidth="1"/>
@@ -839,12 +864,12 @@
         <v>2025</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+    <row r="20" spans="2:7" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
       <c r="B20" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="2:7" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B21" s="1" t="s">
         <v>0</v>
       </c>
@@ -858,7 +883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
         <v>48</v>
       </c>
@@ -872,7 +897,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
         <v>48</v>
       </c>
@@ -886,7 +911,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
         <v>48</v>
       </c>
@@ -900,7 +925,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
         <v>48</v>
       </c>
@@ -912,6 +937,36 @@
       </c>
       <c r="E25" s="3" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="B28" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B29" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="B30" t="s">
+        <v>58</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" t="s">
+        <v>60</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>